<commit_message>
feat: 전압레벨 상향 (154/22.9kV → 345/154kV) — 부하-전압 정합
발전·집전(Bus1·2·6): 154 → 345kV (송전 레벨)
변전·부하(Bus7·3·4·5): 22.9 → 154kV
→ 90MW 부하가 154kV에서 약 340A로 실제 154kV 계통 전류와 유사

- systemModel.ts / python/system_model.py: baseKV 변경
- concepts.html: kV 라벨·계통 설명 전면 갱신 (실제 전압체계 반영)
- 7bus_ems_input_data.xlsx: baseKV 컬럼 갱신
- 전기적 계산값(전압 pu·발전량·손실)은 per-unit이라 불변 (수렴 5회, 발전 93.83MW, 손실 3.83MW 동일)

https://claude.ai/code/session_01KkSrcE6inVX1AKgrva18fe
</commit_message>
<xml_diff>
--- a/7bus_ems_input_data.xlsx
+++ b/7bus_ems_input_data.xlsx
@@ -171,7 +171,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -185,11 +185,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -282,6 +310,8 @@
     <xf numFmtId="0" fontId="4" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -667,6 +697,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -731,7 +762,7 @@
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>154</v>
+        <v>345</v>
       </c>
       <c r="F4" s="6" t="n">
         <v>1.05</v>
@@ -763,7 +794,7 @@
         </is>
       </c>
       <c r="E5" s="8" t="n">
-        <v>154</v>
+        <v>345</v>
       </c>
       <c r="F5" s="8" t="n">
         <v>1.05</v>
@@ -795,7 +826,7 @@
         </is>
       </c>
       <c r="E6" s="9" t="n">
-        <v>154</v>
+        <v>345</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -829,7 +860,7 @@
         </is>
       </c>
       <c r="E7" s="9" t="n">
-        <v>22.9</v>
+        <v>154</v>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
@@ -863,7 +894,7 @@
         </is>
       </c>
       <c r="E8" s="9" t="n">
-        <v>22.9</v>
+        <v>154</v>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
@@ -897,7 +928,7 @@
         </is>
       </c>
       <c r="E9" s="9" t="n">
-        <v>22.9</v>
+        <v>154</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
@@ -931,7 +962,7 @@
         </is>
       </c>
       <c r="E10" s="9" t="n">
-        <v>22.9</v>
+        <v>154</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
@@ -945,6 +976,7 @@
         <v>450</v>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
@@ -996,6 +1028,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1258,6 +1291,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
@@ -1297,12 +1331,17 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>① 부하 설정 (loads)</t>
         </is>
       </c>
+      <c r="B3" s="32" t="n"/>
+      <c r="C3" s="32" t="n"/>
+      <c r="D3" s="32" t="n"/>
+      <c r="E3" s="33" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
@@ -1425,12 +1464,17 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>② 발전기 설정</t>
         </is>
       </c>
+      <c r="B10" s="32" t="n"/>
+      <c r="C10" s="32" t="n"/>
+      <c r="D10" s="32" t="n"/>
+      <c r="E10" s="33" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
@@ -1540,12 +1584,17 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="18" t="inlineStr">
         <is>
           <t>③ 차단기 상태 (breakers)</t>
         </is>
       </c>
+      <c r="B16" s="32" t="n"/>
+      <c r="C16" s="32" t="n"/>
+      <c r="D16" s="32" t="n"/>
+      <c r="E16" s="33" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="19" t="inlineStr">
@@ -1760,12 +1809,19 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>① 모선 해석 결과</t>
         </is>
       </c>
+      <c r="B3" s="32" t="n"/>
+      <c r="C3" s="32" t="n"/>
+      <c r="D3" s="32" t="n"/>
+      <c r="E3" s="32" t="n"/>
+      <c r="F3" s="32" t="n"/>
+      <c r="G3" s="33" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="22" t="inlineStr">
@@ -2049,12 +2105,19 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>② NR 수렴 추이</t>
         </is>
       </c>
+      <c r="B13" s="32" t="n"/>
+      <c r="C13" s="32" t="n"/>
+      <c r="D13" s="32" t="n"/>
+      <c r="E13" s="32" t="n"/>
+      <c r="F13" s="32" t="n"/>
+      <c r="G13" s="33" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="22" t="inlineStr">
@@ -2238,12 +2301,19 @@
       <c r="F19" s="24" t="inlineStr"/>
       <c r="G19" s="24" t="inlineStr"/>
     </row>
+    <row r="20"/>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
           <t>③ 전체 집계</t>
         </is>
       </c>
+      <c r="B21" s="32" t="n"/>
+      <c r="C21" s="32" t="n"/>
+      <c r="D21" s="32" t="n"/>
+      <c r="E21" s="32" t="n"/>
+      <c r="F21" s="32" t="n"/>
+      <c r="G21" s="33" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="28" t="inlineStr">

</xml_diff>